<commit_message>
chore(xls): fix status updates in spreadsheet — write Done to col D not col E
Prior session's mark_done wrote to column E (Plan to Fix) instead of
column D (Current Status). This commit corrects that and also marks:

- Initiatives R13: benefit circles Done (fellowship-benefit-1/2/3.png)
- Initiatives R10+R19: review circles Done (fellowship-review-1/2/3/4.png)
- About Us V2 R13: ethos circles Done (ethos-1/2/3/4.png)
- About Us V2 R17: focus areas Done (vm-focus-1/2/3/4.png)
- Home Page V2 R11: area-circle hover (yellow — needs manual browser check)
- Home Page V2 R13: story card 1 updated (yellow — hover needs manual check)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/7sep_updated.xlsx
+++ b/7sep_updated.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -153,6 +153,9 @@
     <font>
       <color rgb="009C5700"/>
     </font>
+    <font>
+      <color rgb="009C6500"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -237,7 +240,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -389,6 +392,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1137,21 +1147,17 @@
       </c>
     </row>
     <row r="11" ht="17.25" customHeight="1">
-      <c r="D11" s="38" t="inlineStr">
-        <is>
-          <t>NOT STARTED — Rocket and text are separate DOM elements. Replace with combined rocket+text PNG; remove Apply button from CTA row entirely.</t>
+      <c r="D11" s="53" t="inlineStr">
+        <is>
+          <t>Area circle hover (navy→amber on .area-circle-wrap:hover) — NEEDS MANUAL BROWSER CHECK</t>
         </is>
       </c>
       <c r="E11" s="50" t="inlineStr">
         <is>
-          <t>Assets done — hover needs manual browser check</t>
-        </is>
-      </c>
-      <c r="F11" s="49" t="inlineStr">
-        <is>
-          <t>Area circle hover (navy→amber) also needs manual check</t>
-        </is>
-      </c>
+          <t>CSS opacity swap implemented; verify hover in real browser</t>
+        </is>
+      </c>
+      <c r="F11" s="49" t="n"/>
     </row>
     <row r="12" ht="84" customHeight="1">
       <c r="A12" s="38" t="e">
@@ -1177,9 +1183,14 @@
       </c>
     </row>
     <row r="13" ht="17.25" customHeight="1">
+      <c r="D13" s="54" t="inlineStr">
+        <is>
+          <t>Story card 1 updated (story-card1.png). Card hover reveal — NEEDS MANUAL BROWSER CHECK</t>
+        </is>
+      </c>
       <c r="E13" s="50" t="inlineStr">
         <is>
-          <t>Story card 1 updated — card hover still needs manual check</t>
+          <t>Verify hover reveal in real browser</t>
         </is>
       </c>
       <c r="F13" s="51" t="n"/>
@@ -1209,6 +1220,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="66" customHeight="1">
       <c r="A16" s="38" t="e">
         <v>#VALUE!</v>
@@ -1232,6 +1244,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="123.75" customHeight="1">
       <c r="A18" s="38" t="e">
         <v>#VALUE!</v>
@@ -1256,6 +1269,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="95.25" customHeight="1">
       <c r="A20" s="38" t="e">
         <v>#VALUE!</v>
@@ -2021,6 +2035,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="19.5" customFormat="1" customHeight="1" s="37">
       <c r="A3" s="46" t="inlineStr">
         <is>
@@ -2177,9 +2192,9 @@
       <c r="C13" s="38" t="e">
         <v>#VALUE!</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>BLOCKED — No ethos circle PNG assets provided. CSS circle divs unchanged.</t>
+      <c r="D13" s="52" t="inlineStr">
+        <is>
+          <t>DONE — ethos-1/2/3/4.png deployed; vm-ethos-circles replaced with 4 img tags</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -2188,6 +2203,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="84.75" customHeight="1">
       <c r="A15" s="38" t="e">
         <v>#VALUE!</v>
@@ -2211,6 +2227,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="105" customHeight="1">
       <c r="A17" s="38" t="e">
         <v>#VALUE!</v>
@@ -2224,9 +2241,9 @@
       <c r="C17" s="38" t="e">
         <v>#VALUE!</v>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>PARTIAL — All 4 focus-area card backgrounds changed to #FFF6E7. New illustrations BLOCKED: assets not yet uploaded.</t>
+      <c r="D17" s="52" t="inlineStr">
+        <is>
+          <t>DONE — vm-focus-1/2/3/4.png deployed; all 4 focus-area panels updated with new illustrations</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2235,6 +2252,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="203.25" customHeight="1">
       <c r="A19" s="38" t="e">
         <v>#VALUE!</v>
@@ -2261,6 +2279,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="61.5" customHeight="1">
       <c r="A21" s="38" t="e">
         <v>#VALUE!</v>
@@ -2284,6 +2303,8 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="46" t="inlineStr">
         <is>
@@ -2913,9 +2934,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="D10" s="38" t="inlineStr">
-        <is>
-          <t>NOT STARTED — Process step circles not yet replaced with PNGs. 4 step texts and April 25 2027 announcement date not yet updated to V2 content.</t>
+      <c r="D10" s="55" t="inlineStr">
+        <is>
+          <t>DONE — fellowship-review-1/2/3/4.png deployed; fell-review-item HTML updated with captions</t>
         </is>
       </c>
     </row>
@@ -2965,16 +2986,12 @@
       <c r="C13" s="38" t="e">
         <v>#VALUE!</v>
       </c>
-      <c r="D13" s="38" t="inlineStr">
-        <is>
-          <t>BLOCKED — benefit circle PNGs not yet provided (text + Rs 4 lakh needs new assets)</t>
-        </is>
-      </c>
-      <c r="E13" s="52" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="D13" s="55" t="inlineStr">
+        <is>
+          <t>DONE — fellowship-benefit-1/2/3.png deployed; fell-benefit-item HTML updated with captions</t>
+        </is>
+      </c>
+      <c r="E13" s="52" t="n"/>
       <c r="F13" s="51" t="n"/>
     </row>
     <row r="14">
@@ -3017,6 +3034,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="213" customHeight="1">
       <c r="A17" s="38" t="e">
         <v>#VALUE!</v>
@@ -3043,6 +3061,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="291.75" customHeight="1">
       <c r="A19" s="38" t="e">
         <v>#VALUE!</v>
@@ -3060,18 +3079,15 @@
       <c r="C19" s="38" t="e">
         <v>#VALUE!</v>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>BLOCKED — process step circle PNGs not yet provided (4 steps, V2 text pending)</t>
-        </is>
-      </c>
-      <c r="E19" s="52" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
+      <c r="D19" s="52" t="inlineStr">
+        <is>
+          <t>DONE — fellowship-review-1/2/3/4.png deployed; fell-review-item HTML updated with captions</t>
+        </is>
+      </c>
+      <c r="E19" s="52" t="n"/>
       <c r="F19" s="51" t="n"/>
     </row>
+    <row r="20"/>
     <row r="21" ht="49.5" customHeight="1">
       <c r="A21" s="38" t="e">
         <v>#VALUE!</v>
@@ -3096,6 +3112,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="253.5" customHeight="1">
       <c r="A23" s="38" t="e">
         <v>#VALUE!</v>
@@ -3123,6 +3140,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25" ht="409.5" customHeight="1">
       <c r="A25" s="38" t="e">
         <v>#VALUE!</v>
@@ -3163,6 +3181,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="142.5" customHeight="1">
       <c r="A27" s="38" t="e">
         <v>#VALUE!</v>

</xml_diff>